<commit_message>
#4 J9 Connector updated in eSpark and Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/DC-Motor-Driver/Deliverables/BOM/Client BOM.xlsx
+++ b/Design Files/DC-Motor-Driver/Deliverables/BOM/Client BOM.xlsx
@@ -5,21 +5,21 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\manarharake-motordriver\Design Files\DC-Motor-Driver\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9150"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="310">
   <si>
     <t>#</t>
   </si>
@@ -78,9 +78,6 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>LCSC</t>
-  </si>
-  <si>
     <t>C3, C5, C7, C9, C10, C23, C26, C27, C30, C31, C32, C33, C34, C35, C36, C37, C38, C45, C46</t>
   </si>
   <si>
@@ -435,12 +432,6 @@
     <t>Battery button CR2032 SMD Battery Connectors ROHS</t>
   </si>
   <si>
-    <t>MY-2032-10-R</t>
-  </si>
-  <si>
-    <t>MYOUNG</t>
-  </si>
-  <si>
     <t>Male Header</t>
   </si>
   <si>
@@ -946,6 +937,18 @@
   </si>
   <si>
     <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>CR2032-BS-6-1</t>
+  </si>
+  <si>
+    <t>Q&amp;J</t>
+  </si>
+  <si>
+    <t>Sparkfun</t>
+  </si>
+  <si>
+    <t>Quantity 5 Board</t>
   </si>
 </sst>
 </file>
@@ -1579,7 +1582,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:T66"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="28" customWidth="1"/>
@@ -1591,13 +1594,14 @@
     <col min="8" max="8" width="21.42578125" customWidth="1"/>
     <col min="9" max="9" width="8.28515625" customWidth="1"/>
     <col min="10" max="10" width="9" customWidth="1"/>
-    <col min="11" max="11" width="10.42578125" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" customWidth="1"/>
-    <col min="14" max="14" width="16" customWidth="1"/>
-    <col min="15" max="15" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.42578125" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" thickBot="1">
+    <row r="1" spans="1:20" ht="15.75" thickBot="1">
       <c r="A1" s="2"/>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -1610,8 +1614,9 @@
       <c r="J1" s="33"/>
       <c r="K1" s="33"/>
       <c r="L1" s="33"/>
-    </row>
-    <row r="2" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M1" s="33"/>
+    </row>
+    <row r="2" spans="1:20" ht="15.75" thickBot="1">
       <c r="A2" s="2"/>
       <c r="B2" s="5" t="s">
         <v>0</v>
@@ -1641,13 +1646,16 @@
         <v>8</v>
       </c>
       <c r="K2" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="L2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:20">
       <c r="A3" s="2"/>
       <c r="B3" s="7">
         <f t="shared" ref="B3:B64" si="0">ROW(B3)-ROW($B$2)</f>
@@ -1677,10 +1685,14 @@
       <c r="J3" s="9">
         <v>4</v>
       </c>
-      <c r="K3" s="15"/>
-      <c r="L3" s="9"/>
-    </row>
-    <row r="4" spans="1:15" s="1" customFormat="1" ht="36">
+      <c r="K3" s="9">
+        <f>J3*5</f>
+        <v>20</v>
+      </c>
+      <c r="L3" s="15"/>
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" spans="1:20" s="1" customFormat="1" ht="36">
       <c r="A4" s="6"/>
       <c r="B4" s="10">
         <f t="shared" si="0"/>
@@ -1690,32 +1702,40 @@
         <v>11</v>
       </c>
       <c r="D4" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="11" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>21</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J4" s="11">
         <v>19</v>
       </c>
-      <c r="K4" s="16"/>
-      <c r="L4" s="11"/>
-      <c r="N4"/>
+      <c r="K4" s="9">
+        <f t="shared" ref="K4:K64" si="1">J4*5</f>
+        <v>95</v>
+      </c>
+      <c r="L4" s="16"/>
+      <c r="M4" s="11"/>
       <c r="O4"/>
-    </row>
-    <row r="5" spans="1:15" ht="24">
+      <c r="P4"/>
+      <c r="Q4"/>
+      <c r="R4"/>
+      <c r="S4"/>
+      <c r="T4"/>
+    </row>
+    <row r="5" spans="1:20" ht="24">
       <c r="A5" s="2"/>
       <c r="B5" s="7">
         <f t="shared" si="0"/>
@@ -1725,30 +1745,34 @@
         <v>11</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>25</v>
       </c>
       <c r="F5" s="9" t="s">
         <v>14</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J5" s="9">
         <v>9</v>
       </c>
-      <c r="K5" s="15"/>
-      <c r="L5" s="9"/>
-    </row>
-    <row r="6" spans="1:15" ht="24">
+      <c r="K5" s="9">
+        <f t="shared" si="1"/>
+        <v>45</v>
+      </c>
+      <c r="L5" s="15"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" spans="1:20" ht="24">
       <c r="A6" s="2"/>
       <c r="B6" s="10">
         <f t="shared" si="0"/>
@@ -1758,30 +1782,34 @@
         <v>11</v>
       </c>
       <c r="D6" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="11" t="s">
         <v>28</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>29</v>
       </c>
       <c r="F6" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J6" s="11">
         <v>10</v>
       </c>
-      <c r="K6" s="16"/>
-      <c r="L6" s="11"/>
-    </row>
-    <row r="7" spans="1:15">
+      <c r="K6" s="9">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="L6" s="16"/>
+      <c r="M6" s="11"/>
+    </row>
+    <row r="7" spans="1:20">
       <c r="A7" s="2"/>
       <c r="B7" s="7">
         <f t="shared" si="0"/>
@@ -1791,30 +1819,34 @@
         <v>11</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="9" t="s">
         <v>34</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J7" s="9">
         <v>4</v>
       </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="9"/>
-    </row>
-    <row r="8" spans="1:15">
+      <c r="K7" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="L7" s="15"/>
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" spans="1:20">
       <c r="A8" s="2"/>
       <c r="B8" s="10">
         <f t="shared" si="0"/>
@@ -1824,30 +1856,34 @@
         <v>11</v>
       </c>
       <c r="D8" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="F8" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G8" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="I8" s="11" t="s">
         <v>40</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>41</v>
       </c>
       <c r="J8" s="11">
         <v>4</v>
       </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="11"/>
-    </row>
-    <row r="9" spans="1:15">
+      <c r="K8" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="L8" s="16"/>
+      <c r="M8" s="11"/>
+    </row>
+    <row r="9" spans="1:20">
       <c r="A9" s="2"/>
       <c r="B9" s="7">
         <f t="shared" si="0"/>
@@ -1857,30 +1893,34 @@
         <v>11</v>
       </c>
       <c r="D9" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>46</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>47</v>
       </c>
       <c r="J9" s="9">
         <v>1</v>
       </c>
-      <c r="K9" s="15"/>
-      <c r="L9" s="9"/>
-    </row>
-    <row r="10" spans="1:15">
+      <c r="K9" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L9" s="15"/>
+      <c r="M9" s="9"/>
+    </row>
+    <row r="10" spans="1:20">
       <c r="A10" s="2"/>
       <c r="B10" s="10">
         <f t="shared" si="0"/>
@@ -1890,30 +1930,34 @@
         <v>11</v>
       </c>
       <c r="D10" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="G10" s="11" t="s">
+      <c r="H10" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="I10" s="11" t="s">
         <v>51</v>
-      </c>
-      <c r="I10" s="11" t="s">
-        <v>52</v>
       </c>
       <c r="J10" s="11">
         <v>3</v>
       </c>
-      <c r="K10" s="16"/>
-      <c r="L10" s="11"/>
-    </row>
-    <row r="11" spans="1:15">
+      <c r="K10" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L10" s="16"/>
+      <c r="M10" s="11"/>
+    </row>
+    <row r="11" spans="1:20">
       <c r="A11" s="2"/>
       <c r="B11" s="7">
         <f t="shared" si="0"/>
@@ -1923,30 +1967,34 @@
         <v>11</v>
       </c>
       <c r="D11" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="9" t="s">
+      <c r="G11" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="H11" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="9" t="s">
-        <v>57</v>
-      </c>
       <c r="I11" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J11" s="9">
         <v>3</v>
       </c>
-      <c r="K11" s="15"/>
-      <c r="L11" s="9"/>
-    </row>
-    <row r="12" spans="1:15">
+      <c r="K11" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L11" s="15"/>
+      <c r="M11" s="9"/>
+    </row>
+    <row r="12" spans="1:20">
       <c r="A12" s="2"/>
       <c r="B12" s="10">
         <f t="shared" si="0"/>
@@ -1956,30 +2004,34 @@
         <v>11</v>
       </c>
       <c r="D12" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E12" s="11" t="s">
         <v>58</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>59</v>
       </c>
       <c r="F12" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="J12" s="11">
         <v>3</v>
       </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="11"/>
-    </row>
-    <row r="13" spans="1:15">
+      <c r="K12" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L12" s="16"/>
+      <c r="M12" s="11"/>
+    </row>
+    <row r="13" spans="1:20">
       <c r="A13" s="2"/>
       <c r="B13" s="7">
         <f t="shared" si="0"/>
@@ -1989,30 +2041,34 @@
         <v>11</v>
       </c>
       <c r="D13" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="F13" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="G13" s="9" t="s">
         <v>64</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>65</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="J13" s="9">
         <v>3</v>
       </c>
-      <c r="K13" s="15"/>
-      <c r="L13" s="9"/>
-    </row>
-    <row r="14" spans="1:15">
+      <c r="K13" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L13" s="15"/>
+      <c r="M13" s="9"/>
+    </row>
+    <row r="14" spans="1:20">
       <c r="A14" s="2"/>
       <c r="B14" s="10">
         <f t="shared" si="0"/>
@@ -2022,30 +2078,34 @@
         <v>11</v>
       </c>
       <c r="D14" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="F14" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>68</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>69</v>
       </c>
       <c r="H14" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J14" s="11">
         <v>1</v>
       </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="11"/>
-    </row>
-    <row r="15" spans="1:15">
+      <c r="K14" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L14" s="16"/>
+      <c r="M14" s="11"/>
+    </row>
+    <row r="15" spans="1:20">
       <c r="A15" s="2"/>
       <c r="B15" s="7">
         <f t="shared" si="0"/>
@@ -2055,30 +2115,34 @@
         <v>11</v>
       </c>
       <c r="D15" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="F15" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F15" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>73</v>
-      </c>
       <c r="H15" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J15" s="9">
         <v>1</v>
       </c>
-      <c r="K15" s="15"/>
-      <c r="L15" s="9"/>
-    </row>
-    <row r="16" spans="1:15">
+      <c r="K15" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L15" s="15"/>
+      <c r="M15" s="9"/>
+    </row>
+    <row r="16" spans="1:20">
       <c r="A16" s="2"/>
       <c r="B16" s="10">
         <f t="shared" si="0"/>
@@ -2088,30 +2152,34 @@
         <v>11</v>
       </c>
       <c r="D16" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="F16" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="F16" s="11" t="s">
+      <c r="G16" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="H16" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="I16" s="11" t="s">
         <v>78</v>
-      </c>
-      <c r="I16" s="11" t="s">
-        <v>79</v>
       </c>
       <c r="J16" s="11">
         <v>1</v>
       </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="11"/>
-    </row>
-    <row r="17" spans="1:12">
+      <c r="K16" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L16" s="16"/>
+      <c r="M16" s="11"/>
+    </row>
+    <row r="17" spans="1:13">
       <c r="A17" s="2"/>
       <c r="B17" s="7">
         <f t="shared" si="0"/>
@@ -2121,30 +2189,34 @@
         <v>11</v>
       </c>
       <c r="D17" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="F17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="9" t="s">
         <v>81</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>82</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J17" s="9">
         <v>1</v>
       </c>
-      <c r="K17" s="15"/>
-      <c r="L17" s="9"/>
-    </row>
-    <row r="18" spans="1:12">
+      <c r="K17" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L17" s="15"/>
+      <c r="M17" s="9"/>
+    </row>
+    <row r="18" spans="1:13">
       <c r="A18" s="2"/>
       <c r="B18" s="10">
         <f t="shared" si="0"/>
@@ -2154,30 +2226,34 @@
         <v>11</v>
       </c>
       <c r="D18" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="11" t="s">
         <v>84</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>85</v>
       </c>
       <c r="F18" s="11" t="s">
         <v>14</v>
       </c>
       <c r="G18" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" s="11" t="s">
         <v>86</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>87</v>
       </c>
       <c r="J18" s="11">
         <v>1</v>
       </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="11"/>
-    </row>
-    <row r="19" spans="1:12" ht="24">
+      <c r="K18" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L18" s="16"/>
+      <c r="M18" s="11"/>
+    </row>
+    <row r="19" spans="1:13" ht="24">
       <c r="A19" s="2"/>
       <c r="B19" s="7">
         <f t="shared" si="0"/>
@@ -2187,52 +2263,56 @@
         <v>11</v>
       </c>
       <c r="D19" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="9" t="s">
+      <c r="F19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F19" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="G19" s="9" t="s">
+      <c r="H19" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="I19" s="9" t="s">
         <v>91</v>
-      </c>
-      <c r="I19" s="9" t="s">
-        <v>92</v>
       </c>
       <c r="J19" s="9">
         <v>1</v>
       </c>
-      <c r="K19" s="15"/>
-      <c r="L19" s="9"/>
-    </row>
-    <row r="20" spans="1:12" ht="24">
+      <c r="K19" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L19" s="15"/>
+      <c r="M19" s="9"/>
+    </row>
+    <row r="20" spans="1:13" ht="24">
       <c r="A20" s="2"/>
       <c r="B20" s="10">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D20" s="30" t="s">
+        <v>290</v>
+      </c>
+      <c r="E20" s="30" t="s">
+        <v>291</v>
+      </c>
+      <c r="F20" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="G20" s="30" t="s">
+        <v>292</v>
+      </c>
+      <c r="H20" s="30" t="s">
         <v>293</v>
-      </c>
-      <c r="E20" s="30" t="s">
-        <v>294</v>
-      </c>
-      <c r="F20" s="30" t="s">
-        <v>97</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>295</v>
-      </c>
-      <c r="H20" s="30" t="s">
-        <v>296</v>
       </c>
       <c r="I20" s="11" t="s">
         <v>17</v>
@@ -2240,32 +2320,36 @@
       <c r="J20" s="11">
         <v>2</v>
       </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="11"/>
-    </row>
-    <row r="21" spans="1:12" ht="24">
+      <c r="K20" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L20" s="16"/>
+      <c r="M20" s="11"/>
+    </row>
+    <row r="21" spans="1:13" ht="24">
       <c r="A21" s="2"/>
       <c r="B21" s="7">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="H21" s="9" t="s">
-        <v>94</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>17</v>
@@ -2273,32 +2357,36 @@
       <c r="J21" s="9">
         <v>2</v>
       </c>
-      <c r="K21" s="15"/>
-      <c r="L21" s="9"/>
-    </row>
-    <row r="22" spans="1:12" ht="24">
+      <c r="K21" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L21" s="15"/>
+      <c r="M21" s="9"/>
+    </row>
+    <row r="22" spans="1:13" ht="24">
       <c r="A22" s="2"/>
       <c r="B22" s="10">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D22" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="F22" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="G22" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="H22" s="11" t="s">
         <v>102</v>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>103</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>17</v>
@@ -2306,32 +2394,36 @@
       <c r="J22" s="11">
         <v>1</v>
       </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="11"/>
-    </row>
-    <row r="23" spans="1:12">
+      <c r="K22" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L22" s="16"/>
+      <c r="M22" s="11"/>
+    </row>
+    <row r="23" spans="1:13">
       <c r="A23" s="2"/>
       <c r="B23" s="7">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D23" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E23" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="9" t="s">
+      <c r="F23" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="F23" s="9" t="s">
+      <c r="G23" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="G23" s="9" t="s">
+      <c r="H23" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="I23" s="9" t="s">
         <v>17</v>
@@ -2339,32 +2431,36 @@
       <c r="J23" s="9">
         <v>1</v>
       </c>
-      <c r="K23" s="15"/>
-      <c r="L23" s="9"/>
-    </row>
-    <row r="24" spans="1:12" ht="24">
+      <c r="K23" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L23" s="15"/>
+      <c r="M23" s="9"/>
+    </row>
+    <row r="24" spans="1:13" ht="24">
       <c r="A24" s="2"/>
       <c r="B24" s="7">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D24" s="30" t="s">
+        <v>294</v>
+      </c>
+      <c r="E24" s="30" t="s">
+        <v>295</v>
+      </c>
+      <c r="F24" s="30" t="s">
+        <v>296</v>
+      </c>
+      <c r="G24" s="30" t="s">
         <v>297</v>
       </c>
-      <c r="E24" s="30" t="s">
+      <c r="H24" s="30" t="s">
         <v>298</v>
-      </c>
-      <c r="F24" s="30" t="s">
-        <v>299</v>
-      </c>
-      <c r="G24" s="30" t="s">
-        <v>300</v>
-      </c>
-      <c r="H24" s="30" t="s">
-        <v>301</v>
       </c>
       <c r="I24" s="30" t="s">
         <v>17</v>
@@ -2372,32 +2468,36 @@
       <c r="J24" s="30">
         <v>1</v>
       </c>
-      <c r="K24" s="15"/>
-      <c r="L24" s="9"/>
-    </row>
-    <row r="25" spans="1:12" ht="24">
+      <c r="K24" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L24" s="15"/>
+      <c r="M24" s="9"/>
+    </row>
+    <row r="25" spans="1:13" ht="24">
       <c r="A25" s="2"/>
       <c r="B25" s="10">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="E25" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="F25" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="G25" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="G25" s="11" t="s">
+      <c r="H25" s="11" t="s">
         <v>113</v>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>114</v>
       </c>
       <c r="I25" s="9" t="s">
         <v>17</v>
@@ -2405,32 +2505,36 @@
       <c r="J25" s="11">
         <v>1</v>
       </c>
-      <c r="K25" s="16"/>
-      <c r="L25" s="11"/>
-    </row>
-    <row r="26" spans="1:12">
+      <c r="K25" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L25" s="16"/>
+      <c r="M25" s="11"/>
+    </row>
+    <row r="26" spans="1:13">
       <c r="A26" s="2"/>
       <c r="B26" s="7">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="D26" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="E26" s="9" t="s">
+      <c r="F26" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="F26" s="9" t="s">
+      <c r="G26" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="G26" s="9" t="s">
-        <v>119</v>
-      </c>
       <c r="H26" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I26" s="9" t="s">
         <v>17</v>
@@ -2438,26 +2542,30 @@
       <c r="J26" s="9">
         <v>2</v>
       </c>
-      <c r="K26" s="15"/>
-      <c r="L26" s="9"/>
-    </row>
-    <row r="27" spans="1:12" ht="25.5">
+      <c r="K26" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L26" s="15"/>
+      <c r="M26" s="9"/>
+    </row>
+    <row r="27" spans="1:13" ht="25.5">
       <c r="A27" s="2"/>
       <c r="B27" s="10">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D27" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="D27" s="13" t="s">
-        <v>121</v>
       </c>
       <c r="E27" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G27" s="13" t="s">
         <v>17</v>
@@ -2466,74 +2574,82 @@
         <v>17</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J27" s="13">
         <v>6</v>
       </c>
-      <c r="K27" s="13"/>
-      <c r="L27" s="17" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" ht="25.5">
+      <c r="K27" s="9">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="L27" s="13"/>
+      <c r="M27" s="17" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" ht="25.5">
       <c r="A28" s="2"/>
       <c r="B28" s="7">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C28" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="D28" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="E28" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="F28" s="14" t="s">
         <v>127</v>
-      </c>
-      <c r="F28" s="14" t="s">
-        <v>128</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>17</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I28" s="14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J28" s="14">
         <v>1</v>
       </c>
-      <c r="K28" s="13"/>
-      <c r="L28" s="17" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12">
+      <c r="K28" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L28" s="13"/>
+      <c r="M28" s="17" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13">
       <c r="A29" s="2"/>
       <c r="B29" s="10">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="D29" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="E29" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="F29" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="F29" s="11" t="s">
+      <c r="G29" s="11" t="s">
         <v>132</v>
       </c>
-      <c r="G29" s="11" t="s">
+      <c r="H29" s="11" t="s">
         <v>133</v>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>134</v>
       </c>
       <c r="I29" s="11" t="s">
         <v>17</v>
@@ -2541,32 +2657,36 @@
       <c r="J29" s="11">
         <v>1</v>
       </c>
-      <c r="K29" s="16"/>
-      <c r="L29" s="11"/>
-    </row>
-    <row r="30" spans="1:12" ht="24">
+      <c r="K29" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L29" s="16"/>
+      <c r="M29" s="11"/>
+    </row>
+    <row r="30" spans="1:13" ht="24">
       <c r="A30" s="2"/>
       <c r="B30" s="7">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="E30" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="E30" s="9" t="s">
-        <v>137</v>
-      </c>
       <c r="F30" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="G30" s="9" t="s">
-        <v>138</v>
+        <v>131</v>
+      </c>
+      <c r="G30" s="30" t="s">
+        <v>306</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>139</v>
+        <v>307</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>17</v>
@@ -2574,32 +2694,36 @@
       <c r="J30" s="9">
         <v>1</v>
       </c>
-      <c r="K30" s="15"/>
-      <c r="L30" s="9"/>
-    </row>
-    <row r="31" spans="1:12">
+      <c r="K30" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L30" s="15"/>
+      <c r="M30" s="9"/>
+    </row>
+    <row r="31" spans="1:13">
       <c r="A31" s="2"/>
       <c r="B31" s="10">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="E31" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F31" s="11" t="s">
         <v>140</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="E31" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="F31" s="11" t="s">
-        <v>143</v>
       </c>
       <c r="G31" s="11">
         <v>8266292</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>17</v>
@@ -2607,131 +2731,147 @@
       <c r="J31" s="11">
         <v>1</v>
       </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="11"/>
-    </row>
-    <row r="32" spans="1:12">
+      <c r="K31" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L31" s="16"/>
+      <c r="M31" s="11"/>
+    </row>
+    <row r="32" spans="1:13">
       <c r="A32" s="2"/>
       <c r="B32" s="7">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F32" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="D32" s="9" t="s">
+      <c r="G32" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="E32" s="9" t="s">
+      <c r="H32" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="I32" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="H32" s="9" t="s">
-        <v>40</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>150</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
-      <c r="K32" s="15"/>
-      <c r="L32" s="9"/>
-    </row>
-    <row r="33" spans="1:12">
+      <c r="K32" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L32" s="15"/>
+      <c r="M32" s="9"/>
+    </row>
+    <row r="33" spans="1:13">
       <c r="A33" s="2"/>
       <c r="B33" s="10">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D33" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="H33" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="E33" s="11" t="s">
+      <c r="I33" s="11" t="s">
         <v>152</v>
-      </c>
-      <c r="F33" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="G33" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="H33" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="I33" s="11" t="s">
-        <v>155</v>
       </c>
       <c r="J33" s="11">
         <v>1</v>
       </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="11"/>
-    </row>
-    <row r="34" spans="1:12" ht="36">
+      <c r="K33" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L33" s="16"/>
+      <c r="M33" s="11"/>
+    </row>
+    <row r="34" spans="1:13" ht="36">
       <c r="A34" s="2"/>
       <c r="B34" s="7">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D34" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="H34" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="E34" s="9" t="s">
+      <c r="I34" s="9" t="s">
         <v>157</v>
-      </c>
-      <c r="F34" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="H34" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="I34" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
       </c>
-      <c r="K34" s="15"/>
-      <c r="L34" s="9"/>
-    </row>
-    <row r="35" spans="1:12" ht="24">
+      <c r="K34" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L34" s="15"/>
+      <c r="M34" s="9"/>
+    </row>
+    <row r="35" spans="1:13" ht="24">
       <c r="A35" s="2"/>
       <c r="B35" s="10">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
       <c r="C35" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="F35" s="11" t="s">
         <v>161</v>
       </c>
-      <c r="D35" s="11" t="s">
+      <c r="G35" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="E35" s="11" t="s">
+      <c r="H35" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="G35" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="H35" s="11" t="s">
-        <v>166</v>
       </c>
       <c r="I35" s="11" t="s">
         <v>17</v>
@@ -2739,32 +2879,36 @@
       <c r="J35" s="11">
         <v>1</v>
       </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="11"/>
-    </row>
-    <row r="36" spans="1:12" ht="48">
+      <c r="K35" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L35" s="16"/>
+      <c r="M35" s="11"/>
+    </row>
+    <row r="36" spans="1:13" ht="48">
       <c r="A36" s="2"/>
       <c r="B36" s="7">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D36" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="G36" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="E36" s="9" t="s">
+      <c r="H36" s="9" t="s">
         <v>168</v>
-      </c>
-      <c r="F36" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="G36" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="H36" s="9" t="s">
-        <v>171</v>
       </c>
       <c r="I36" s="11" t="s">
         <v>17</v>
@@ -2772,26 +2916,30 @@
       <c r="J36" s="9">
         <v>1</v>
       </c>
-      <c r="K36" s="15"/>
-      <c r="L36" s="9"/>
-    </row>
-    <row r="37" spans="1:12">
+      <c r="K36" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L36" s="15"/>
+      <c r="M36" s="9"/>
+    </row>
+    <row r="37" spans="1:13">
       <c r="A37" s="2"/>
       <c r="B37" s="10">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E37" s="13" t="s">
         <v>17</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="G37" s="13" t="s">
         <v>17</v>
@@ -2805,32 +2953,36 @@
       <c r="J37" s="13">
         <v>1</v>
       </c>
-      <c r="K37" s="13"/>
+      <c r="K37" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
       <c r="L37" s="13"/>
-    </row>
-    <row r="38" spans="1:12" ht="36">
+      <c r="M37" s="13"/>
+    </row>
+    <row r="38" spans="1:13" ht="36">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
       <c r="C38" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="F38" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="G38" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="E38" s="9" t="s">
+      <c r="H38" s="9" t="s">
         <v>177</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="G38" s="9" t="s">
-        <v>179</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>180</v>
       </c>
       <c r="I38" s="11" t="s">
         <v>17</v>
@@ -2838,32 +2990,36 @@
       <c r="J38" s="9">
         <v>1</v>
       </c>
-      <c r="K38" s="15"/>
-      <c r="L38" s="9"/>
-    </row>
-    <row r="39" spans="1:12" ht="48">
+      <c r="K38" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L38" s="15"/>
+      <c r="M38" s="9"/>
+    </row>
+    <row r="39" spans="1:13" ht="48">
       <c r="A39" s="2"/>
       <c r="B39" s="10">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D39" s="11" t="s">
+        <v>178</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F39" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="G39" s="11" t="s">
         <v>181</v>
       </c>
-      <c r="E39" s="11" t="s">
+      <c r="H39" s="11" t="s">
         <v>182</v>
-      </c>
-      <c r="F39" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="G39" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="H39" s="11" t="s">
-        <v>185</v>
       </c>
       <c r="I39" s="11" t="s">
         <v>17</v>
@@ -2871,395 +3027,443 @@
       <c r="J39" s="11">
         <v>1</v>
       </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="11"/>
-    </row>
-    <row r="40" spans="1:12">
+      <c r="K39" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L39" s="16"/>
+      <c r="M39" s="11"/>
+    </row>
+    <row r="40" spans="1:13">
       <c r="A40" s="2"/>
       <c r="B40" s="7">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
       <c r="C40" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="F40" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="D40" s="9" t="s">
+      <c r="G40" s="9" t="s">
         <v>187</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="F40" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="G40" s="9" t="s">
-        <v>190</v>
       </c>
       <c r="H40" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I40" s="9" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J40" s="9">
         <v>2</v>
       </c>
-      <c r="K40" s="15"/>
-      <c r="L40" s="9"/>
-    </row>
-    <row r="41" spans="1:12">
+      <c r="K40" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L40" s="15"/>
+      <c r="M40" s="9"/>
+    </row>
+    <row r="41" spans="1:13">
       <c r="A41" s="2"/>
       <c r="B41" s="10">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D41" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="F41" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="G41" s="11" t="s">
         <v>192</v>
-      </c>
-      <c r="E41" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="F41" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="G41" s="11" t="s">
-        <v>195</v>
       </c>
       <c r="H41" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="J41" s="11">
         <v>2</v>
       </c>
-      <c r="K41" s="16"/>
-      <c r="L41" s="11"/>
-    </row>
-    <row r="42" spans="1:12">
+      <c r="K41" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L41" s="16"/>
+      <c r="M41" s="11"/>
+    </row>
+    <row r="42" spans="1:13">
       <c r="A42" s="2"/>
       <c r="B42" s="7">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D42" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F42" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="G42" s="9" t="s">
         <v>197</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="F42" s="9" t="s">
-        <v>199</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="H42" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="J42" s="9">
         <v>5</v>
       </c>
-      <c r="K42" s="15"/>
-      <c r="L42" s="9"/>
-    </row>
-    <row r="43" spans="1:12">
+      <c r="K42" s="9">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="L42" s="15"/>
+      <c r="M42" s="9"/>
+    </row>
+    <row r="43" spans="1:13">
       <c r="A43" s="2"/>
       <c r="B43" s="10">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F43" s="11" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H43" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="J43" s="11">
         <v>2</v>
       </c>
-      <c r="K43" s="16"/>
-      <c r="L43" s="11"/>
-    </row>
-    <row r="44" spans="1:12">
+      <c r="K43" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L43" s="16"/>
+      <c r="M43" s="11"/>
+    </row>
+    <row r="44" spans="1:13">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E44" s="9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I44" s="9" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="J44" s="9">
         <v>1</v>
       </c>
-      <c r="K44" s="15"/>
-      <c r="L44" s="9"/>
-    </row>
-    <row r="45" spans="1:12">
+      <c r="K44" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L44" s="15"/>
+      <c r="M44" s="9"/>
+    </row>
+    <row r="45" spans="1:13">
       <c r="A45" s="2"/>
       <c r="B45" s="10">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F45" s="11" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="H45" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="J45" s="11">
         <v>3</v>
       </c>
-      <c r="K45" s="16"/>
-      <c r="L45" s="11"/>
-    </row>
-    <row r="46" spans="1:12" ht="36">
+      <c r="K45" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L45" s="16"/>
+      <c r="M45" s="11"/>
+    </row>
+    <row r="46" spans="1:13" ht="36">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D46" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="G46" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="H46" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="I46" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>217</v>
-      </c>
-      <c r="H46" s="9" t="s">
-        <v>218</v>
-      </c>
-      <c r="I46" s="9" t="s">
-        <v>219</v>
       </c>
       <c r="J46" s="9">
         <v>3</v>
       </c>
-      <c r="K46" s="15"/>
-      <c r="L46" s="9"/>
-    </row>
-    <row r="47" spans="1:12">
+      <c r="K46" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L46" s="15"/>
+      <c r="M46" s="9"/>
+    </row>
+    <row r="47" spans="1:13">
       <c r="A47" s="2"/>
       <c r="B47" s="10">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F47" s="11" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G47" s="11" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="H47" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I47" s="11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="J47" s="11">
         <v>1</v>
       </c>
-      <c r="K47" s="16"/>
-      <c r="L47" s="11"/>
-    </row>
-    <row r="48" spans="1:12">
+      <c r="K47" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L47" s="16"/>
+      <c r="M47" s="11"/>
+    </row>
+    <row r="48" spans="1:13">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E48" s="9" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="H48" s="9" t="s">
         <v>16</v>
       </c>
       <c r="I48" s="9" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="J48" s="9">
         <v>1</v>
       </c>
-      <c r="K48" s="15"/>
-      <c r="L48" s="9"/>
-    </row>
-    <row r="49" spans="1:15">
+      <c r="K48" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L48" s="15"/>
+      <c r="M48" s="9"/>
+    </row>
+    <row r="49" spans="1:20">
       <c r="A49" s="2"/>
       <c r="B49" s="10">
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="F49" s="11" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="H49" s="11" t="s">
         <v>16</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J49" s="11">
         <v>1</v>
       </c>
-      <c r="K49" s="16"/>
-      <c r="L49" s="11"/>
-    </row>
-    <row r="50" spans="1:15">
+      <c r="K49" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L49" s="16"/>
+      <c r="M49" s="11"/>
+    </row>
+    <row r="50" spans="1:20">
       <c r="A50" s="2"/>
       <c r="B50" s="10">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C50" s="31" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D50" s="30" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="E50" s="30" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="H50" s="30" t="s">
         <v>16</v>
       </c>
       <c r="I50" s="30" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
       </c>
-      <c r="K50" s="15"/>
-      <c r="L50" s="9"/>
-    </row>
-    <row r="51" spans="1:15">
+      <c r="K50" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L50" s="15"/>
+      <c r="M50" s="9"/>
+    </row>
+    <row r="51" spans="1:20">
       <c r="A51" s="2"/>
       <c r="B51" s="7">
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
       <c r="C51" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="G51" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="H51" s="9" t="s">
         <v>233</v>
-      </c>
-      <c r="E51" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="H51" s="9" t="s">
-        <v>236</v>
       </c>
       <c r="I51" s="9" t="s">
         <v>17</v>
@@ -3267,32 +3471,36 @@
       <c r="J51" s="9">
         <v>2</v>
       </c>
-      <c r="K51" s="15"/>
-      <c r="L51" s="9"/>
-    </row>
-    <row r="52" spans="1:15" s="1" customFormat="1">
+      <c r="K51" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="L51" s="15"/>
+      <c r="M51" s="9"/>
+    </row>
+    <row r="52" spans="1:20" s="1" customFormat="1">
       <c r="A52" s="6"/>
       <c r="B52" s="10">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
       <c r="C52" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F52" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="G52" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="E52" s="11" t="s">
+      <c r="H52" s="11" t="s">
         <v>239</v>
-      </c>
-      <c r="F52" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="G52" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="H52" s="11" t="s">
-        <v>242</v>
       </c>
       <c r="I52" s="11" t="s">
         <v>17</v>
@@ -3300,34 +3508,42 @@
       <c r="J52" s="11">
         <v>1</v>
       </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="11"/>
-      <c r="N52"/>
+      <c r="K52" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L52" s="16"/>
+      <c r="M52" s="11"/>
       <c r="O52"/>
-    </row>
-    <row r="53" spans="1:15">
+      <c r="P52"/>
+      <c r="Q52"/>
+      <c r="R52"/>
+      <c r="S52"/>
+      <c r="T52"/>
+    </row>
+    <row r="53" spans="1:20">
       <c r="A53" s="2"/>
       <c r="B53" s="7">
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D53" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="G53" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="E53" s="9" t="s">
+      <c r="H53" s="9" t="s">
         <v>244</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="H53" s="9" t="s">
-        <v>247</v>
       </c>
       <c r="I53" s="9" t="s">
         <v>17</v>
@@ -3335,32 +3551,36 @@
       <c r="J53" s="9">
         <v>1</v>
       </c>
-      <c r="K53" s="15"/>
-      <c r="L53" s="9"/>
-    </row>
-    <row r="54" spans="1:15">
+      <c r="K53" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L53" s="15"/>
+      <c r="M53" s="9"/>
+    </row>
+    <row r="54" spans="1:20">
       <c r="A54" s="2"/>
       <c r="B54" s="10">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D54" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="E54" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="F54" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="G54" s="11" t="s">
         <v>248</v>
       </c>
-      <c r="E54" s="11" t="s">
+      <c r="H54" s="11" t="s">
         <v>249</v>
-      </c>
-      <c r="F54" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="G54" s="11" t="s">
-        <v>251</v>
-      </c>
-      <c r="H54" s="11" t="s">
-        <v>252</v>
       </c>
       <c r="I54" s="11" t="s">
         <v>17</v>
@@ -3368,32 +3588,36 @@
       <c r="J54" s="11">
         <v>1</v>
       </c>
-      <c r="K54" s="16"/>
-      <c r="L54" s="11"/>
-    </row>
-    <row r="55" spans="1:15">
+      <c r="K54" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L54" s="16"/>
+      <c r="M54" s="11"/>
+    </row>
+    <row r="55" spans="1:20">
       <c r="A55" s="2"/>
       <c r="B55" s="7">
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D55" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="G55" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="E55" s="9" t="s">
+      <c r="H55" s="9" t="s">
         <v>254</v>
-      </c>
-      <c r="F55" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>257</v>
       </c>
       <c r="I55" s="9" t="s">
         <v>17</v>
@@ -3401,219 +3625,247 @@
       <c r="J55" s="9">
         <v>1</v>
       </c>
-      <c r="K55" s="15"/>
-      <c r="L55" s="9"/>
-    </row>
-    <row r="56" spans="1:15">
+      <c r="K55" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L55" s="15"/>
+      <c r="M55" s="9"/>
+    </row>
+    <row r="56" spans="1:20">
       <c r="A56" s="2"/>
       <c r="B56" s="10">
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D56" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="E56" s="11" t="s">
+        <v>256</v>
+      </c>
+      <c r="F56" s="11" t="s">
+        <v>257</v>
+      </c>
+      <c r="G56" s="11" t="s">
         <v>258</v>
       </c>
-      <c r="E56" s="11" t="s">
+      <c r="H56" s="11" t="s">
         <v>259</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="G56" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="H56" s="11" t="s">
-        <v>262</v>
       </c>
       <c r="I56" s="11"/>
       <c r="J56" s="11">
         <v>3</v>
       </c>
-      <c r="K56" s="16"/>
-      <c r="L56" s="11"/>
-    </row>
-    <row r="57" spans="1:15">
+      <c r="K56" s="9">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="L56" s="16"/>
+      <c r="M56" s="11"/>
+    </row>
+    <row r="57" spans="1:20">
       <c r="A57" s="2"/>
       <c r="B57" s="7">
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D57" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="G57" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="E57" s="9" t="s">
+      <c r="H57" s="9" t="s">
         <v>264</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>266</v>
-      </c>
-      <c r="H57" s="9" t="s">
-        <v>267</v>
       </c>
       <c r="I57" s="9"/>
       <c r="J57" s="9">
         <v>1</v>
       </c>
-      <c r="K57" s="15"/>
-      <c r="L57" s="9"/>
-    </row>
-    <row r="58" spans="1:15">
+      <c r="K57" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L57" s="15"/>
+      <c r="M57" s="9"/>
+    </row>
+    <row r="58" spans="1:20">
       <c r="A58" s="2"/>
       <c r="B58" s="10">
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D58" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="E58" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="F58" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="G58" s="11" t="s">
         <v>268</v>
       </c>
-      <c r="E58" s="11" t="s">
+      <c r="H58" s="11" t="s">
         <v>269</v>
-      </c>
-      <c r="F58" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="G58" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="H58" s="11" t="s">
-        <v>272</v>
       </c>
       <c r="I58" s="11"/>
       <c r="J58" s="11">
         <v>1</v>
       </c>
-      <c r="K58" s="16"/>
-      <c r="L58" s="11"/>
-    </row>
-    <row r="59" spans="1:15">
+      <c r="K58" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L58" s="16"/>
+      <c r="M58" s="11"/>
+    </row>
+    <row r="59" spans="1:20">
       <c r="A59" s="2"/>
       <c r="B59" s="7">
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D59" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="G59" s="9" t="s">
         <v>273</v>
       </c>
-      <c r="E59" s="9" t="s">
-        <v>274</v>
-      </c>
-      <c r="F59" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>276</v>
-      </c>
       <c r="H59" s="9" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="I59" s="9"/>
       <c r="J59" s="9">
         <v>1</v>
       </c>
-      <c r="K59" s="15"/>
-      <c r="L59" s="9"/>
-    </row>
-    <row r="60" spans="1:15" ht="36">
+      <c r="K59" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L59" s="15"/>
+      <c r="M59" s="9"/>
+    </row>
+    <row r="60" spans="1:20" ht="36">
       <c r="A60" s="2"/>
       <c r="B60" s="10">
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
       <c r="C60" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="D60" s="11" t="s">
+        <v>275</v>
+      </c>
+      <c r="E60" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="F60" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="G60" s="11" t="s">
         <v>277</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="H60" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="E60" s="11" t="s">
+      <c r="I60" s="11" t="s">
         <v>279</v>
-      </c>
-      <c r="F60" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="G60" s="11" t="s">
-        <v>280</v>
-      </c>
-      <c r="H60" s="11" t="s">
-        <v>281</v>
-      </c>
-      <c r="I60" s="11" t="s">
-        <v>282</v>
       </c>
       <c r="J60" s="11">
         <v>1</v>
       </c>
-      <c r="K60" s="16"/>
-      <c r="L60" s="11"/>
-    </row>
-    <row r="61" spans="1:15" ht="24">
+      <c r="K60" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L60" s="16"/>
+      <c r="M60" s="11"/>
+    </row>
+    <row r="61" spans="1:20" ht="24">
       <c r="A61" s="2"/>
       <c r="B61" s="7">
         <f t="shared" si="0"/>
         <v>59</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D61" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>281</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="H61" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="E61" s="9" t="s">
+      <c r="I61" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="F61" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="I61" s="9" t="s">
-        <v>287</v>
       </c>
       <c r="J61" s="9">
         <v>1</v>
       </c>
-      <c r="K61" s="15"/>
-      <c r="L61" s="9"/>
-    </row>
-    <row r="62" spans="1:15">
+      <c r="K61" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L61" s="15"/>
+      <c r="M61" s="9"/>
+    </row>
+    <row r="62" spans="1:20">
       <c r="A62" s="2"/>
       <c r="B62" s="7">
         <f t="shared" si="0"/>
         <v>60</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D62" s="9" t="s">
         <v>17</v>
       </c>
       <c r="E62" s="9" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="F62" s="11" t="s">
         <v>17</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="H62" s="9" t="s">
         <v>17</v>
@@ -3622,31 +3874,35 @@
       <c r="J62" s="9">
         <v>5</v>
       </c>
-      <c r="K62" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="L62" s="9"/>
-    </row>
-    <row r="63" spans="1:15">
+      <c r="K62" s="9">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="L62" s="15" t="s">
+        <v>308</v>
+      </c>
+      <c r="M62" s="9"/>
+    </row>
+    <row r="63" spans="1:20">
       <c r="A63" s="2"/>
       <c r="B63" s="7">
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D63" s="32" t="s">
         <v>17</v>
       </c>
       <c r="E63" s="32" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F63" s="11" t="s">
         <v>17</v>
       </c>
       <c r="G63" s="32" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="H63" s="9" t="s">
         <v>17</v>
@@ -3657,37 +3913,45 @@
       <c r="J63" s="9">
         <v>1</v>
       </c>
-      <c r="K63" s="15" t="s">
-        <v>308</v>
-      </c>
-      <c r="L63" s="9"/>
-    </row>
-    <row r="64" spans="1:15" ht="15.75" thickBot="1">
+      <c r="K63" s="9">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="L63" s="15" t="s">
+        <v>305</v>
+      </c>
+      <c r="M63" s="9"/>
+    </row>
+    <row r="64" spans="1:20" ht="15.75" thickBot="1">
       <c r="A64" s="2"/>
       <c r="B64" s="7">
         <f t="shared" si="0"/>
         <v>62</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D64" s="9"/>
       <c r="E64" s="9" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F64" s="11"/>
       <c r="G64" s="9" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="H64" s="9"/>
       <c r="I64" s="9"/>
       <c r="J64" s="9">
         <v>6</v>
       </c>
-      <c r="K64" s="15"/>
-      <c r="L64" s="9"/>
-    </row>
-    <row r="65" spans="1:12" ht="19.5" thickBot="1">
+      <c r="K64" s="9">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="L64" s="15"/>
+      <c r="M64" s="9"/>
+    </row>
+    <row r="65" spans="1:13" ht="19.5" thickBot="1">
       <c r="A65" s="2"/>
       <c r="B65" s="18"/>
       <c r="C65" s="19"/>
@@ -3698,10 +3962,11 @@
       <c r="H65" s="22"/>
       <c r="I65" s="23"/>
       <c r="J65" s="23"/>
-      <c r="K65" s="29"/>
-      <c r="L65" s="34"/>
-    </row>
-    <row r="66" spans="1:12" ht="19.5" thickBot="1">
+      <c r="K65" s="23"/>
+      <c r="L65" s="29"/>
+      <c r="M65" s="34"/>
+    </row>
+    <row r="66" spans="1:13" ht="19.5" thickBot="1">
       <c r="A66" s="2"/>
       <c r="B66" s="24"/>
       <c r="C66" s="25"/>
@@ -3712,17 +3977,18 @@
       <c r="H66" s="27"/>
       <c r="I66" s="27"/>
       <c r="J66" s="27"/>
-      <c r="K66" s="29"/>
-      <c r="L66" s="35"/>
+      <c r="K66" s="27"/>
+      <c r="L66" s="29"/>
+      <c r="M66" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="I1:L1"/>
-    <mergeCell ref="L65:L66"/>
+    <mergeCell ref="I1:M1"/>
+    <mergeCell ref="M65:M66"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K62" r:id="rId1"/>
-    <hyperlink ref="K63" r:id="rId2"/>
+    <hyperlink ref="L63" r:id="rId1"/>
+    <hyperlink ref="L62" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>